<commit_message>
added v3 testing documentation
</commit_message>
<xml_diff>
--- a/agent_testing_results.xlsx
+++ b/agent_testing_results.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stephen.gaffney\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C83C4170-77B7-4EA1-8C9A-0694CDAD5C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFCC61B3-2063-47DD-9E4A-EBEA925AD9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V1 Testing" sheetId="1" r:id="rId1"/>
     <sheet name="V2 Testing" sheetId="2" r:id="rId2"/>
+    <sheet name="V3 Testing" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="107">
   <si>
     <t>#</t>
   </si>
@@ -37,12 +38,18 @@
     <t>Result</t>
   </si>
   <si>
+    <t>Fail Description</t>
+  </si>
+  <si>
     <t>Remember my dog's name is Dani, a Shih Tzu</t>
   </si>
   <si>
     <t>Fail - blank response, no tool call shown</t>
   </si>
   <si>
+    <t>Blank-response bug. Model failed to generate any output or tool call on that turn. Possibly a race condition on the very first inference call after model load. Retried later with an OK repsonse</t>
+  </si>
+  <si>
     <t>Calculator: 384 * 17 + 92</t>
   </si>
   <si>
@@ -85,12 +92,18 @@
     <t>Fail - declined, claimed no way to fetch facts</t>
   </si>
   <si>
+    <t>Model didn't recognize it could just answer from its own trained knowledge; treated it as needing an external source it didn't have. Thought it needed a new web search or something of the like.</t>
+  </si>
+  <si>
     <t>"Let's do the random fun fact" (retry)</t>
   </si>
   <si>
     <t>Partial - got a real fact, but fabricated a tool call first</t>
   </si>
   <si>
+    <t>Invented a file path (/usr/local/path/facts.txt) that doesn't exist. Output also had Chinese text mid-sentence, which is a known multilingual-leakage quirk in smaller Qwen models that have been trained on more than just English.</t>
+  </si>
+  <si>
     <t>Explain REST API</t>
   </si>
   <si>
@@ -139,12 +152,18 @@
     <t>Fail - tool correctly errored ("Unsupported expression"), but model answered "4" anyway</t>
   </si>
   <si>
+    <t>Model overrode its own tool's failure with a guess from training knowledge, presenting it with identical confidence to the verified results next to it. The most concerning pattern here, since there's no visible signal distinguishing a tool-verified answer from a guess/hallucination.</t>
+  </si>
+  <si>
     <t>"What time is it / what day"</t>
   </si>
   <si>
     <t>Fail - blank final response after tool calls</t>
   </si>
   <si>
+    <t>Blank-response bug again. The expected retry warning line wasn't visible in the transcript, so it is unclear if the retry logic happened or if this is a gap in detection. I will retest and check again tomorrow.</t>
+  </si>
+  <si>
     <t>Remember favorite color (blue) + meeting Tuesday</t>
   </si>
   <si>
@@ -166,18 +185,27 @@
     <t>Fail - tool correctly refused (multiple matches, nothing deleted) but model claimed it removed the memory</t>
   </si>
   <si>
+    <t>Model narrated a false outcome contradicting its own tool's actual return value. It said an action succeeded when the tool explicitly reported it didn't happen.</t>
+  </si>
+  <si>
     <t>User replies "5" to disambiguate</t>
   </si>
   <si>
     <t>Fail - no tool call fired at all, yet model claimed the memory was removed</t>
   </si>
   <si>
+    <t>Complete fabrication/hallucination. The model treated a bare number as resolved without actually issuing the corresponding forget call. Confirmed false by the next recall, which showed both entries were still present.</t>
+  </si>
+  <si>
     <t>User flags the inconsistency</t>
   </si>
   <si>
     <t>Partial - recall was accurate, but the model's spoken summary only listed 3 of 6 real entries</t>
   </si>
   <si>
+    <t>Summary drifted from the actual tool output it had just received, which likely was blending in stale info from earlier turns rather than re-reading the fresh recall result carefully.</t>
+  </si>
+  <si>
     <t>"Forget that I own a spaceship" (no match)</t>
   </si>
   <si>
@@ -187,9 +215,21 @@
     <t>User repeats the green-grass deletion request</t>
   </si>
   <si>
+    <t>Pass (finally executed correctly after multiple human retries)</t>
+  </si>
+  <si>
+    <t>Took two extra user corrections to actually fire not a failure of the tool itself, but shows the model needed explicit re-prompting rather than self-correcting from the earlier contradiction.</t>
+  </si>
+  <si>
     <t>"Forget entry 2"</t>
   </si>
   <si>
+    <t>Fail - deleted index [1] (the imperial units fact) instead of index [2] (the Python fact)</t>
+  </si>
+  <si>
+    <t>Off-by-one confusion which is due to counting "entry 2" as the second item in casual 1-based counting rather than matching the literal [2] label shown by the recall tool output immediately prior.</t>
+  </si>
+  <si>
     <t>Read test_notes.txt (exists)</t>
   </si>
   <si>
@@ -208,56 +248,6 @@
     <t>Final: dog's name + imperial/metric preference</t>
   </si>
   <si>
-    <t>Fail Description</t>
-  </si>
-  <si>
-    <t>Blank-response bug. Model failed to generate any output or tool call on that turn. Possibly a race condition on the very first inference call after model load. Retried later with an OK repsonse</t>
-  </si>
-  <si>
-    <t>Model didn't recognize it could just answer from its own trained knowledge; treated it as needing an external source it didn't have. Thought it needed a new web search or something of the like.</t>
-  </si>
-  <si>
-    <t>Invented a file path (/usr/local/path/facts.txt) that doesn't exist. Output also had Chinese text mid-sentence, which is a known multilingual-leakage quirk in smaller Qwen models that have been trained on more than just English.</t>
-  </si>
-  <si>
-    <t>Model overrode its own tool's failure with a guess from training knowledge, presenting it with identical confidence to the verified results next to it. The most concerning pattern here, since there's no visible signal distinguishing a tool-verified answer from a guess/hallucination.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Blank-response bug again. The expected retry warning line wasn't visible in the transcript, so it is unclear if the retry logic happened or if this is a gap in detection. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>I will retest and check again tomorrow.</t>
-    </r>
-  </si>
-  <si>
-    <t>Model narrated a false outcome contradicting its own tool's actual return value. It said an action succeeded when the tool explicitly reported it didn't happen.</t>
-  </si>
-  <si>
-    <t>Complete fabrication/hallucination. The model treated a bare number as resolved without actually issuing the corresponding forget call. Confirmed false by the next recall, which showed both entries were still present.</t>
-  </si>
-  <si>
-    <t>Summary drifted from the actual tool output it had just received, which likely was blending in stale info from earlier turns rather than re-reading the fresh recall result carefully.</t>
-  </si>
-  <si>
-    <t>Took two extra user corrections to actually fire not a failure of the tool itself, but shows the model needed explicit re-prompting rather than self-correcting from the earlier contradiction.</t>
-  </si>
-  <si>
-    <t>Pass (finally executed correctly after multiple human retries)</t>
-  </si>
-  <si>
-    <t>Fail - deleted index [1] (the imperial units fact) instead of index [2] (the Python fact)</t>
-  </si>
-  <si>
-    <t>Off-by-one confusion which is due to counting "entry 2" as the second item in casual 1-based counting rather than matching the literal [2] label shown by the recall tool output immediately prior.</t>
-  </si>
-  <si>
     <t>Fail - answered "you prefer imperial units" but that fact had already been deleted in test 14 (this is probably not an error of not deleting that fact, but rather because the model had that info from earlier in the chat not memory.)</t>
   </si>
   <si>
@@ -265,13 +255,106 @@
   </si>
   <si>
     <t>Pass - confirmed true persistent memory even after Spyder relaunch</t>
+  </si>
+  <si>
+    <t>Why It May Have Failed / Notes</t>
+  </si>
+  <si>
+    <t>Current time / day of week</t>
+  </si>
+  <si>
+    <t>Unit conversion: km-to-mile, F-to-C, kg-to-lb + mismatched-category error (kg-to-mile)</t>
+  </si>
+  <si>
+    <t>All four valid conversions correct; mismatched-category case returned the intended clean error rather than a fabricated number.</t>
+  </si>
+  <si>
+    <t>Remember/recall, including cross-session recall from v2's memory.json</t>
+  </si>
+  <si>
+    <t>Confirms memory.json format carried over cleanly between script versions.</t>
+  </si>
+  <si>
+    <t>Two-step forget - confirm path (stage, then "yes")</t>
+  </si>
+  <si>
+    <t>Confirmation step worked as designed. Not independently re-verified against recall in this round -- worth a quick double-check next time given v2's history of false success claims.</t>
+  </si>
+  <si>
+    <t>Two-step forget - decline path (stage, then "no")</t>
+  </si>
+  <si>
+    <t>Correctly left the entry untouched.</t>
+  </si>
+  <si>
+    <t>Forget - ambiguous match (multiple entries)</t>
+  </si>
+  <si>
+    <t>Untested</t>
+  </si>
+  <si>
+    <t>Forget - no match (nonexistent fact)</t>
+  </si>
+  <si>
+    <t>Partial</t>
+  </si>
+  <si>
+    <t>Notes: add_note + list_notes</t>
+  </si>
+  <si>
+    <t>Read file: success + missing-file error</t>
+  </si>
+  <si>
+    <t>Blank-response fix: two chained-tool-call prompts</t>
+  </si>
+  <si>
+    <t>Sliding window stress test ("what did I ask 10 messages ago")</t>
+  </si>
+  <si>
+    <t>Honestly reported lack of access rather than fabricating an answer.</t>
+  </si>
+  <si>
+    <t>Cross-session persistence (full restart)</t>
+  </si>
+  <si>
+    <t>confirm_forget misuse (called with nothing staged)</t>
+  </si>
+  <si>
+    <t>Blank-response retry safeguard (unprompted observation)</t>
+  </si>
+  <si>
+    <t>At one point where a blank reply would previously have occurred silently (per v2 behavior), the safeguard fired correctly and returned the intended fallback message asking the user to rephrase, rather than an empty response.</t>
+  </si>
+  <si>
+    <t>Startup sanity check - all 10 skills loaded</t>
+  </si>
+  <si>
+    <t>Calculator: normal expressions + divide by 0 + sqrt(16) edge case</t>
+  </si>
+  <si>
+    <t>Unlike v2, the sqrt case no longer produced a silent hallucinated override. Correct error handling this time.</t>
+  </si>
+  <si>
+    <t>First response was unrelated/off-topic rather than the correct "no match" message, but importantly, no fabricated success like the v2 bug. Second attempt (after user re-prompted) gave the correct error. It is worth investigating why the first attempt didn't route to the tool correctly, so I will retest.</t>
+  </si>
+  <si>
+    <t>add_note itself works correctly because notes.json contains accurate, correctly timestamped entries. However, retrieval is unreliable: when asked "what notes have I saved," the model calls recall instead of list_notes, returning the wrong data source. Need to look into why this is happening and how we can make it clear for which skill to use.</t>
+  </si>
+  <si>
+    <t>Tool-call chaining itself worked structurally (no blank replies) for both prompts. However, the notes-related prompt still called recall instead of list_notes, same root cause as test 10, not a chaining failure.</t>
+  </si>
+  <si>
+    <t>memory.json persistence fully confirmed correct. notes.json also persisted correctly on my computer with accurate data, but the same recall-vs-list_notes confusion from tests 10/12 appeared again during retrieval after restart.</t>
+  </si>
+  <si>
+    <t>Pushed back to Monday</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,25 +375,21 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -326,19 +405,25 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4E4"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFCE4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -369,7 +454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -386,6 +471,9 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -398,8 +486,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,7 +516,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFE7E6E6"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -684,21 +772,21 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>61</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -706,10 +794,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2"/>
     </row>
@@ -718,10 +806,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2"/>
     </row>
@@ -730,10 +818,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2"/>
     </row>
@@ -742,10 +830,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2"/>
     </row>
@@ -754,10 +842,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" s="2"/>
     </row>
@@ -766,10 +854,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D8" s="2"/>
     </row>
@@ -778,10 +866,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2"/>
     </row>
@@ -790,39 +878,39 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="50" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -830,10 +918,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D13" s="2"/>
     </row>
@@ -842,10 +930,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D14" s="2"/>
     </row>
@@ -854,10 +942,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2"/>
     </row>
@@ -866,10 +954,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D16" s="2"/>
     </row>
@@ -900,277 +988,525 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="7">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="7">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="7">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="7">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="7">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="7">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="6">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="7">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="7">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="7">
+        <v>16</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="7">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7">
+        <v>18</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7">
+        <v>19</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" ht="50" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="6">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="6">
-        <v>4</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="6">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="6">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="6">
-        <v>7</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="6">
-        <v>8</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="6">
-        <v>9</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="6">
-        <v>10</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="6">
-        <v>11</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="6">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="6">
-        <v>13</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="6">
-        <v>14</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="6">
-        <v>15</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="6">
-        <v>16</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="6">
-        <v>17</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" spans="1:4" ht="50" x14ac:dyDescent="0.35">
-      <c r="A21" s="6">
-        <v>18</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="25" x14ac:dyDescent="0.35">
-      <c r="A22" s="6">
-        <v>19</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>75</v>
       </c>
       <c r="D22" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="65" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>98</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
v3.2: fix calculator sqrt/abs/round, add_note corruption, forget punctuation matching.
</commit_message>
<xml_diff>
--- a/agent_testing_results.xlsx
+++ b/agent_testing_results.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stephen.gaffney\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765AF69C-C2F3-4DC5-AEE5-D87C5F6B7812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{444B55ED-54A1-4D99-87FC-F25F2E3D72B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V1 Testing" sheetId="7" r:id="rId1"/>
     <sheet name="V2 Testing" sheetId="6" r:id="rId2"/>
     <sheet name="V3 Testing" sheetId="5" r:id="rId3"/>
     <sheet name="V3.1 Testing" sheetId="4" r:id="rId4"/>
+    <sheet name="V3.2 Testing" sheetId="8" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="153">
   <si>
     <t>#</t>
   </si>
@@ -424,6 +425,69 @@
   </si>
   <si>
     <t>Divide-by-zero handled correctly. sqrt(16) still shows the same v2/v3 pattern: the tool correctly errored ("Unsupported expression"), but the model answered "4" anyway from its own knowledge, with the same confidence as verified results. Not something v3.1 fixed, so I'm not surprised it still exists.</t>
+  </si>
+  <si>
+    <t>Chained tool calls: date+notes, miles+long-term-memory</t>
+  </si>
+  <si>
+    <t>Functionally correct, though this turn is where the fabricated forget narrative from test 12 resurfaced unprompted.</t>
+  </si>
+  <si>
+    <t>confirm_forget misuse ("yes" with nothing actually staged)</t>
+  </si>
+  <si>
+    <t>Forget - ambiguous "green" match + decline</t>
+  </si>
+  <si>
+    <t>Forget - dog fact ("Dani") + confirm yes</t>
+  </si>
+  <si>
+    <t>Forget - imperial units preference</t>
+  </si>
+  <si>
+    <t>"What do you have saved in memory?" (asked again right after 2 facts were saved)</t>
+  </si>
+  <si>
+    <t>v3.2 fix confirmed working: both notes saved as clean plain strings, no malformed nested objects this time. notes.json data is accurate.</t>
+  </si>
+  <si>
+    <t>Remember/recall (initial save)</t>
+  </si>
+  <si>
+    <t>Unit conversion: km-to-mile, F-to-C, kg-to-lb, kg-to-mile (mismatched)</t>
+  </si>
+  <si>
+    <t>Calculator: sqrt, abs, round, normal expressions, divide-by-zero</t>
+  </si>
+  <si>
+    <t>v3.2 fix confirmed working: sqrt(16), abs(-7), and round(3.14159, 2) all executed correctly via the tool itself. No override with a guessed answer. Divide-by-zero and standard arithmetic also correct.</t>
+  </si>
+  <si>
+    <t>All four answers were numerically correct, but convert_units was never actually called this session. The model used calculator with manually hardcoded conversion constants instead (e.g. '10 * 0.621371'). The kg-to-mile mismatch was also caught correctly, but via the model's reasoning rather than the tool's built-in category-mismatch error. Not a v3.2 regression (convert_units itself wasn't edited), but worth noting the tool went completely unused despite being available and correct.</t>
+  </si>
+  <si>
+    <t>Falsely claimed "Currently, there are no facts or preferences saved" which directly contradicted the 2 facts that had just been saved and correctly recalled moments earlier. No recall tool call was made this time; the model appears to have answered from a confused read of recent context rather than checking ground truth.</t>
+  </si>
+  <si>
+    <t>New failure, different from the v3.1 punctuation bug: the model passed a paraphrased search key ('prefer_metric') instead of a literal snippet of the saved text ('I prefer imperial units over metric'). Since matching is substring-based (even with v3.2's punctuation normalization), a paraphrase that doesn't appear in the saved fact will never match. This is a real limitation of substring matching in general, not something v3.2's specific fix targeted.</t>
+  </si>
+  <si>
+    <t>This time the model passed an actual substring ("Dani") correctly staged, correctly deleted on confirmation, verified accurate via later recall.</t>
+  </si>
+  <si>
+    <t>Correctly listed both matches and never staged/deleted anything throughout (memory stayed safe). However, it took two attempts to correctly process the decline "don't forget either" was misread as still wanting to proceed, and only the more explicit "Neither" was understood correctly.</t>
+  </si>
+  <si>
+    <t>The v3.1/v3.2 fix went well here: correctly reported no match without asking for yes/no confirmation immediately afterward, as intended.</t>
+  </si>
+  <si>
+    <t>Rather than asking for unwarranted confirmation (the old bug) or correctly saying nothing is pending, the model fabricated an entirely fictional "staged for deletion" state with no tool call at all. This persisted into the next, unrelated request (reading a file), resurfacing unprompted ("Would you like me to proceed with forgetting this entry now?") before finally being dropped after an explicit second "no."</t>
+  </si>
+  <si>
+    <t>"Today's date + notes" correctly chained get_current_time and list_notes. "5 miles to km + what's in long-term memory" only called calculator for the conversion (see test 4) and never called recall. It falsely claimed memory was empty despite 3 facts existing at the time (confirmed by the relaunch chat's later recall), and appears to have mislabeled stale notes-list context as the answer instead.</t>
+  </si>
+  <si>
+    <t>Both facts and notes persisted correctly across a full restart, and the very first message correctly chained both recall and list_notes in one turn with fully accurate data for both stores.</t>
   </si>
 </sst>
 </file>
@@ -1833,4 +1897,252 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{835390F1-E6D0-4229-9849-3EE4813EA510}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="75" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="50" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="50" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="62.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v3.3: fix forget paraphrase matching, convert_units bypass, tool-dropping; document new confirm_forget over-triggering regression -- Testing Results uploaded with priorities for 3.4 -- Updates README with v3.3 architecture, fix-by-fix results, and known-bugs list for v3.4.
</commit_message>
<xml_diff>
--- a/agent_testing_results.xlsx
+++ b/agent_testing_results.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stephen.gaffney\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stephen.gaffney\Desktop\AI Research - July 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{444B55ED-54A1-4D99-87FC-F25F2E3D72B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE851F2B-CD29-4ED3-B742-D6519F100EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V1 Testing" sheetId="7" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="V3 Testing" sheetId="5" r:id="rId3"/>
     <sheet name="V3.1 Testing" sheetId="4" r:id="rId4"/>
     <sheet name="V3.2 Testing" sheetId="8" r:id="rId5"/>
+    <sheet name="V3.3 Testing" sheetId="9" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="174">
   <si>
     <t>#</t>
   </si>
@@ -488,6 +489,69 @@
   </si>
   <si>
     <t>Both facts and notes persisted correctly across a full restart, and the very first message correctly chained both recall and list_notes in one turn with fully accurate data for both stores.</t>
+  </si>
+  <si>
+    <t>Excellent result, both facts and notes persisted correctly, and the very first message after a full restart correctly chained both tools with fully accurate data.</t>
+  </si>
+  <si>
+    <t>Honestly said no instead of making up an answer.</t>
+  </si>
+  <si>
+    <t>Correct this time. Both multi-part prompts correctly fired both needed tools (get_current_time+list_notes; convert_units+recall), resolving the selective tool-dropping seen in earlier versions, at least for these two cases.</t>
+  </si>
+  <si>
+    <t>Functionally correct, though a minor new confabulation appeared: after reading test_notes.txt, the assistant unprompted called it "a timestamped note from your log" and offered to remove it, mixing file-reading output with the memory/forget system without being asked.</t>
+  </si>
+  <si>
+    <t>The v3.3 intercept fired exactly as designed here -- deterministic "nothing pending" response, no fabrication. Notably, this is the SAME mechanism that caused the regression in test 5 -- it works correctly for its intended trigger but over-fires on unrelated affirmative replies.</t>
+  </si>
+  <si>
+    <t>confirm_forget misuse ("yes" with nothing staged, in proper isolated context)</t>
+  </si>
+  <si>
+    <t>Correctly reported no match without asking for confirmation.</t>
+  </si>
+  <si>
+    <t>Correctly listed both matches, and this time correctly recognized "Don't forget either" as a decline on the FIRST attempt (improvement over v3.2, which needed two tries). Minor wording imprecision in the response ("no memory matching your request was found," when matches were in fact found but declined), functionally correct, just slightly confusing phrasing.</t>
+  </si>
+  <si>
+    <t>Forget - ambiguous "green" match + decline ("Don't forget either")</t>
+  </si>
+  <si>
+    <t>Core v3.3 fix confirmed working exactly as designed: the compressed/paraphrased target correctly matched "I prefer imperial units over metric" via the new word-subset matching tier, staged and deleted correctly, verified accurate via follow-up recall.</t>
+  </si>
+  <si>
+    <t>Forget - paraphrase matching ("prefer_metric")</t>
+  </si>
+  <si>
+    <t>Correctly staged (matched on a partial multi-word target) and deleted on confirmation.</t>
+  </si>
+  <si>
+    <t>Forget - dog fact, confirm path</t>
+  </si>
+  <si>
+    <t>Clean plain-string notes (v3.2 fix holding up), and correct list_notes retrieval once the phrasing was unambiguous.</t>
+  </si>
+  <si>
+    <t>Add notes (add_note x2) + retrieve via clearly-phrased "What notes have I saved?"</t>
+  </si>
+  <si>
+    <t>Two distinct issues: (a) the first two asks incorrectly triggered a list_notes tool call instead of recall, answering a facts question with notes data ("no notes saved yet") (b) A third ask later got a confidently false "no facts saved" answer despite 2 real facts existing at the time</t>
+  </si>
+  <si>
+    <t>"What do you have saved in memory?" (asked 3 times across the session)</t>
+  </si>
+  <si>
+    <t>New Bug: from the v3.3 confirm_forget intercept: the model added an unprompted "Is this correct?" after each remember call. Replying "yes" (a normal, unrelated affirmative) triggered the bare-yes/no intercept meant only for forget confirmations, producing the canned "There's nothing pending to confirm" response, which was completely off-topic for what was actually being confirmed. Happened on both remember calls. The intercept is scoped too broad: it treats any bare yes/no as forget-related regardless of what the model just asked.</t>
+  </si>
+  <si>
+    <t>Remember (dog, imperial units) + model's own "Is this correct?" follow-up</t>
+  </si>
+  <si>
+    <t>v3.3 fix confirmed working: convert_units was actually called for all three valid conversions this time. The mismatched kg-to-mile case still didn't invoke the tool itself, but the model correctly reasoned through the mismatch conversationally rather than fabricating a number.</t>
+  </si>
+  <si>
+    <t>All correct, consistent with v3.2's confirmed fix holding up.</t>
   </si>
 </sst>
 </file>
@@ -2145,4 +2209,254 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD4B36E9-A62F-4973-8597-402E010C14EF}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="75" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="50" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>